<commit_message>
chore: Merapihkan button di manajemen data siswa dan guru
</commit_message>
<xml_diff>
--- a/public/templates/Template_Import_Guru.xlsx
+++ b/public/templates/Template_Import_Guru.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ardi\Documents\Kuliah\SEM 6\Propen\SIABSEN\FE\siabsen-app-fe\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{705BD871-451B-4075-A901-9082EE6E41F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E70315-11F7-4B95-A0C8-1E0EE5507B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C0B7A6CC-4030-424C-9199-5BA98C300436}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Nama Pegawai</t>
   </si>
@@ -48,19 +48,22 @@
     <t>Mata Pelajaran</t>
   </si>
   <si>
-    <t>Perempuan</t>
-  </si>
-  <si>
-    <t>Biologi</t>
-  </si>
-  <si>
-    <t>STAFF</t>
-  </si>
-  <si>
-    <t>TEST</t>
-  </si>
-  <si>
     <t>NUPTK</t>
+  </si>
+  <si>
+    <t>Masukkan &lt;GURU&gt; atau &lt;STAF&gt;</t>
+  </si>
+  <si>
+    <t>Masukkan &lt;Laki-laki&gt; atau &lt;Perempuan&gt;</t>
+  </si>
+  <si>
+    <t>Masukkan &lt;Nama_Matpel&gt;</t>
+  </si>
+  <si>
+    <t>Masukkan &lt;Nama Guru/Staf&gt;</t>
+  </si>
+  <si>
+    <t>Masukkan &lt;16 digit NUPTK/NIP&gt;</t>
   </si>
 </sst>
 </file>
@@ -429,16 +432,16 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.08984375" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="13.7265625" customWidth="1"/>
+    <col min="1" max="1" width="27.08984375" customWidth="1"/>
+    <col min="2" max="2" width="25.6328125" customWidth="1"/>
+    <col min="3" max="3" width="35.1796875" customWidth="1"/>
+    <col min="4" max="4" width="30.6328125" customWidth="1"/>
     <col min="5" max="5" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -454,20 +457,20 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>9090909090909090</v>
+      <c r="A2" t="s">
+        <v>9</v>
       </c>
       <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>